<commit_message>
feat: transform Decision Tree into Location & Site Selection Optimizer
</commit_message>
<xml_diff>
--- a/data/RoastLab_All_Datasets.xlsx
+++ b/data/RoastLab_All_Datasets.xlsx
@@ -8,11 +8,11 @@
   </bookViews>
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="1. Cold Brew Demand (LR)" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="2. Bean Recommendations (NB)" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="2. Bean Origin (NB)" sheetId="2" state="visible" r:id="rId2"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="3. Drinks Catalog (KNN)" sheetId="3" state="visible" r:id="rId3"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="3. Taste Profiles (KNN)" sheetId="4" state="visible" r:id="rId4"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="4. Reviews Sentiment (SVM)" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="5. Bean Quiz (Decision Tree)" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="5. Site Selection (DT)" sheetId="6" state="visible" r:id="rId6"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="6. Roast Telemetry (ANN)" sheetId="7" state="visible" r:id="rId7"/>
   </sheets>
   <definedNames/>
@@ -25605,358 +25605,870 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D16"/>
+  <dimension ref="A1:F27"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>body</t>
+          <t>foot_traffic</t>
         </is>
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>acidity</t>
+          <t>rent_budget</t>
         </is>
       </c>
       <c r="C1" t="inlineStr">
         <is>
-          <t>flavor_profile</t>
+          <t>dwell_time</t>
         </is>
       </c>
       <c r="D1" t="inlineStr">
         <is>
-          <t>recommended_bean</t>
+          <t>parking_access</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>space_capacity</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>store_format</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Light/Tea-like</t>
+          <t>Heavy Transit &amp; Office Commuters</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>High/Bright</t>
+          <t>High / Prime Downtown ($$$$)</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Fruity/Floral</t>
+          <t>Grab-&amp;-Go (&lt; 10 mins)</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Ethiopian Yirgacheffe</t>
+          <t>Transit Hub / Walk-Up Only (Zero Parking)</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>Micro Space (&lt; 40 sqm)</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>Downtown CBD Express Kiosk</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Light/Tea-like</t>
+          <t>Heavy Transit &amp; Office Commuters</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Balanced</t>
+          <t>High / Prime Downtown ($$$$)</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Fruity/Floral</t>
+          <t>Grab-&amp;-Go (&lt; 10 mins)</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Ethiopian Yirgacheffe</t>
+          <t>Street Parking &amp; Shared Lot</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>Micro Space (&lt; 40 sqm)</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>Downtown CBD Express Kiosk</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Medium/Smooth</t>
+          <t>Heavy Transit &amp; Office Commuters</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>High/Bright</t>
+          <t>Moderate / Urban Commercial ($$)</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Fruity/Floral</t>
+          <t>Grab-&amp;-Go (&lt; 10 mins)</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Ethiopian Yirgacheffe</t>
+          <t>Transit Hub / Walk-Up Only (Zero Parking)</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>Micro Space (&lt; 40 sqm)</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>Downtown CBD Express Kiosk</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Medium/Smooth</t>
+          <t>Heavy Transit &amp; Office Commuters</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>High/Bright</t>
+          <t>High / Prime Downtown ($$$$)</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Earthy/Spicy</t>
+          <t>Grab-&amp;-Go (&lt; 10 mins)</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Kenyan AA</t>
+          <t>Transit Hub / Walk-Up Only (Zero Parking)</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>Standard Lounge (80 - 150 sqm)</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>Downtown CBD Express Kiosk</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Light/Tea-like</t>
+          <t>Moderate Student &amp; Academic</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>High/Bright</t>
+          <t>Moderate / Urban Commercial ($$)</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Earthy/Spicy</t>
+          <t>Extended Study &amp; Work (&gt; 60 mins)</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>Kenyan AA</t>
+          <t>Transit Hub / Walk-Up Only (Zero Parking)</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>Standard Lounge (80 - 150 sqm)</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>University Campus Study Lounge</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Medium/Smooth</t>
+          <t>Moderate Student &amp; Academic</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Balanced</t>
+          <t>Moderate / Urban Commercial ($$)</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Chocolatey/Nutty</t>
+          <t>Extended Study &amp; Work (&gt; 60 mins)</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>Colombian Supremo</t>
+          <t>Street Parking &amp; Shared Lot</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>Standard Lounge (80 - 150 sqm)</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>University Campus Study Lounge</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Medium/Smooth</t>
+          <t>Moderate Student &amp; Academic</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Low/Mild</t>
+          <t>Economical / Low Overhead ($)</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Chocolatey/Nutty</t>
+          <t>Extended Study &amp; Work (&gt; 60 mins)</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>Colombian Supremo</t>
+          <t>Transit Hub / Walk-Up Only (Zero Parking)</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>Standard Lounge (80 - 150 sqm)</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>University Campus Study Lounge</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Light/Tea-like</t>
+          <t>Moderate Student &amp; Academic</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Balanced</t>
+          <t>Moderate / Urban Commercial ($$)</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Chocolatey/Nutty</t>
+          <t>Extended Study &amp; Work (&gt; 60 mins)</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>Colombian Supremo</t>
+          <t>Street Parking &amp; Shared Lot</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>Spacious Destination (&gt; 200 sqm)</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>University Campus Study Lounge</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Medium/Smooth</t>
+          <t>Moderate Student &amp; Academic</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>High/Bright</t>
+          <t>Economical / Low Overhead ($)</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Chocolatey/Nutty</t>
+          <t>Extended Study &amp; Work (&gt; 60 mins)</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>Guatemalan Antigua</t>
+          <t>Street Parking &amp; Shared Lot</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>Standard Lounge (80 - 150 sqm)</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>University Campus Study Lounge</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Heavy/Syrupy</t>
+          <t>Neighborhood Residents &amp; Families</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>High/Bright</t>
+          <t>Moderate / Urban Commercial ($$)</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Chocolatey/Nutty</t>
+          <t>Social Dine-In &amp; Brunch (30 - 60 mins)</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>Guatemalan Antigua</t>
+          <t>Street Parking &amp; Shared Lot</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>Spacious Destination (&gt; 200 sqm)</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>Suburban Community Roastery &amp; Patio</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Heavy/Syrupy</t>
+          <t>Neighborhood Residents &amp; Families</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Low/Mild</t>
+          <t>Economical / Low Overhead ($)</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Earthy/Spicy</t>
+          <t>Social Dine-In &amp; Brunch (30 - 60 mins)</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>Sumatra Mandheling</t>
+          <t>Street Parking &amp; Shared Lot</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>Spacious Destination (&gt; 200 sqm)</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>Suburban Community Roastery &amp; Patio</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Heavy/Syrupy</t>
+          <t>Neighborhood Residents &amp; Families</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Balanced</t>
+          <t>Moderate / Urban Commercial ($$)</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Earthy/Spicy</t>
+          <t>Social Dine-In &amp; Brunch (30 - 60 mins)</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>Sumatra Mandheling</t>
+          <t>Street Parking &amp; Shared Lot</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>Standard Lounge (80 - 150 sqm)</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>Suburban Community Roastery &amp; Patio</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Medium/Smooth</t>
+          <t>Neighborhood Residents &amp; Families</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Low/Mild</t>
+          <t>Moderate / Urban Commercial ($$)</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Earthy/Spicy</t>
+          <t>Extended Study &amp; Work (&gt; 60 mins)</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>Sumatra Mandheling</t>
+          <t>Street Parking &amp; Shared Lot</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>Spacious Destination (&gt; 200 sqm)</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>Suburban Community Roastery &amp; Patio</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Heavy/Syrupy</t>
+          <t>Neighborhood Residents &amp; Families</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Low/Mild</t>
+          <t>Economical / Low Overhead ($)</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Chocolatey/Nutty</t>
+          <t>Social Dine-In &amp; Brunch (30 - 60 mins)</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>Brazilian Santos</t>
+          <t>Dedicated Drive-Thru &amp; Ample Parking</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>Spacious Destination (&gt; 200 sqm)</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>Suburban Community Roastery &amp; Patio</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Heavy/Syrupy</t>
+          <t>Low Pedestrian / High Vehicular Flow</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Balanced</t>
+          <t>Economical / Low Overhead ($)</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Chocolatey/Nutty</t>
+          <t>Grab-&amp;-Go (&lt; 10 mins)</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>Brazilian Santos</t>
+          <t>Dedicated Drive-Thru &amp; Ample Parking</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>Standard Lounge (80 - 150 sqm)</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>Highway Commuter Drive-Thru Express</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>Low Pedestrian / High Vehicular Flow</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>Moderate / Urban Commercial ($$)</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>Grab-&amp;-Go (&lt; 10 mins)</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>Dedicated Drive-Thru &amp; Ample Parking</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>Standard Lounge (80 - 150 sqm)</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>Highway Commuter Drive-Thru Express</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>Low Pedestrian / High Vehicular Flow</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>Economical / Low Overhead ($)</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>Grab-&amp;-Go (&lt; 10 mins)</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>Dedicated Drive-Thru &amp; Ample Parking</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>Micro Space (&lt; 40 sqm)</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>Highway Commuter Drive-Thru Express</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>Low Pedestrian / High Vehicular Flow</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>Economical / Low Overhead ($)</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>Social Dine-In &amp; Brunch (30 - 60 mins)</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>Dedicated Drive-Thru &amp; Ample Parking</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>Standard Lounge (80 - 150 sqm)</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>Highway Commuter Drive-Thru Express</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>Weekend Leisure &amp; Tourists</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>High / Prime Downtown ($$$$)</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>Social Dine-In &amp; Brunch (30 - 60 mins)</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>Transit Hub / Walk-Up Only (Zero Parking)</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>Spacious Destination (&gt; 200 sqm)</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>Arts &amp; Heritage Flagship Tasting Room</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>Weekend Leisure &amp; Tourists</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>Moderate / Urban Commercial ($$)</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>Social Dine-In &amp; Brunch (30 - 60 mins)</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>Street Parking &amp; Shared Lot</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>Spacious Destination (&gt; 200 sqm)</t>
+        </is>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>Arts &amp; Heritage Flagship Tasting Room</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>Weekend Leisure &amp; Tourists</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>High / Prime Downtown ($$$$)</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>Extended Study &amp; Work (&gt; 60 mins)</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>Street Parking &amp; Shared Lot</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>Spacious Destination (&gt; 200 sqm)</t>
+        </is>
+      </c>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>Arts &amp; Heritage Flagship Tasting Room</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>Weekend Leisure &amp; Tourists</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>Moderate / Urban Commercial ($$)</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>Extended Study &amp; Work (&gt; 60 mins)</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>Transit Hub / Walk-Up Only (Zero Parking)</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>Spacious Destination (&gt; 200 sqm)</t>
+        </is>
+      </c>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>Arts &amp; Heritage Flagship Tasting Room</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>Heavy Transit &amp; Office Commuters</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>Economical / Low Overhead ($)</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>Grab-&amp;-Go (&lt; 10 mins)</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>Street Parking &amp; Shared Lot</t>
+        </is>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>Micro Space (&lt; 40 sqm)</t>
+        </is>
+      </c>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>Corporate Business Park Micro-Lobby</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>Heavy Transit &amp; Office Commuters</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>Economical / Low Overhead ($)</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>Grab-&amp;-Go (&lt; 10 mins)</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>Transit Hub / Walk-Up Only (Zero Parking)</t>
+        </is>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>Micro Space (&lt; 40 sqm)</t>
+        </is>
+      </c>
+      <c r="F25" t="inlineStr">
+        <is>
+          <t>Corporate Business Park Micro-Lobby</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>Moderate Student &amp; Academic</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>Economical / Low Overhead ($)</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>Grab-&amp;-Go (&lt; 10 mins)</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>Transit Hub / Walk-Up Only (Zero Parking)</t>
+        </is>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>Micro Space (&lt; 40 sqm)</t>
+        </is>
+      </c>
+      <c r="F26" t="inlineStr">
+        <is>
+          <t>Corporate Business Park Micro-Lobby</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>Heavy Transit &amp; Office Commuters</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>Economical / Low Overhead ($)</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>Moderate Stay (15 - 45 mins)</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>Street Parking &amp; Shared Lot</t>
+        </is>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>Micro Space (&lt; 40 sqm)</t>
+        </is>
+      </c>
+      <c r="F27" t="inlineStr">
+        <is>
+          <t>Corporate Business Park Micro-Lobby</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat: simplify Decision Tree to binary Yes/No coffee shop location feasibility
</commit_message>
<xml_diff>
--- a/data/RoastLab_All_Datasets.xlsx
+++ b/data/RoastLab_All_Datasets.xlsx
@@ -12,7 +12,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="3. Drinks Catalog (KNN)" sheetId="3" state="visible" r:id="rId3"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="3. Taste Profiles (KNN)" sheetId="4" state="visible" r:id="rId4"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="4. Reviews Sentiment (SVM)" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="5. Site Selection (DT)" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="5. Location Feasibility (DT)" sheetId="6" state="visible" r:id="rId6"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="6. Roast Telemetry (ANN)" sheetId="7" state="visible" r:id="rId7"/>
   </sheets>
   <definedNames/>
@@ -25605,7 +25605,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F27"/>
+  <dimension ref="A1:E18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -25616,859 +25616,481 @@
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>rent_budget</t>
+          <t>rent_cost</t>
         </is>
       </c>
       <c r="C1" t="inlineStr">
         <is>
-          <t>dwell_time</t>
+          <t>competition</t>
         </is>
       </c>
       <c r="D1" t="inlineStr">
         <is>
-          <t>parking_access</t>
+          <t>accessibility</t>
         </is>
       </c>
       <c r="E1" t="inlineStr">
         <is>
-          <t>space_capacity</t>
-        </is>
-      </c>
-      <c r="F1" t="inlineStr">
-        <is>
-          <t>store_format</t>
+          <t>open_coffee_shop</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Heavy Transit &amp; Office Commuters</t>
+          <t>High</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>High / Prime Downtown ($$$$)</t>
+          <t>Affordable</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Grab-&amp;-Go (&lt; 10 mins)</t>
+          <t>Low</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Transit Hub / Walk-Up Only (Zero Parking)</t>
+          <t>Good</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>Micro Space (&lt; 40 sqm)</t>
-        </is>
-      </c>
-      <c r="F2" t="inlineStr">
-        <is>
-          <t>Downtown CBD Express Kiosk</t>
+          <t>Yes</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Heavy Transit &amp; Office Commuters</t>
+          <t>High</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>High / Prime Downtown ($$$$)</t>
+          <t>Affordable</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Grab-&amp;-Go (&lt; 10 mins)</t>
+          <t>High</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Street Parking &amp; Shared Lot</t>
+          <t>Good</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>Micro Space (&lt; 40 sqm)</t>
-        </is>
-      </c>
-      <c r="F3" t="inlineStr">
-        <is>
-          <t>Downtown CBD Express Kiosk</t>
+          <t>Yes</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Heavy Transit &amp; Office Commuters</t>
+          <t>High</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Moderate / Urban Commercial ($$)</t>
+          <t>Moderate</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Grab-&amp;-Go (&lt; 10 mins)</t>
+          <t>Low</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Transit Hub / Walk-Up Only (Zero Parking)</t>
+          <t>Good</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>Micro Space (&lt; 40 sqm)</t>
-        </is>
-      </c>
-      <c r="F4" t="inlineStr">
-        <is>
-          <t>Downtown CBD Express Kiosk</t>
+          <t>Yes</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Heavy Transit &amp; Office Commuters</t>
+          <t>High</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>High / Prime Downtown ($$$$)</t>
+          <t>Moderate</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Grab-&amp;-Go (&lt; 10 mins)</t>
+          <t>High</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Transit Hub / Walk-Up Only (Zero Parking)</t>
+          <t>Good</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>Standard Lounge (80 - 150 sqm)</t>
-        </is>
-      </c>
-      <c r="F5" t="inlineStr">
-        <is>
-          <t>Downtown CBD Express Kiosk</t>
+          <t>Yes</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Moderate Student &amp; Academic</t>
+          <t>High</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Moderate / Urban Commercial ($$)</t>
+          <t>Expensive</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Extended Study &amp; Work (&gt; 60 mins)</t>
+          <t>Low</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>Transit Hub / Walk-Up Only (Zero Parking)</t>
+          <t>Good</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>Standard Lounge (80 - 150 sqm)</t>
-        </is>
-      </c>
-      <c r="F6" t="inlineStr">
-        <is>
-          <t>University Campus Study Lounge</t>
+          <t>Yes</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Moderate Student &amp; Academic</t>
+          <t>High</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Moderate / Urban Commercial ($$)</t>
+          <t>Expensive</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Extended Study &amp; Work (&gt; 60 mins)</t>
+          <t>High</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>Street Parking &amp; Shared Lot</t>
+          <t>Good</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>Standard Lounge (80 - 150 sqm)</t>
-        </is>
-      </c>
-      <c r="F7" t="inlineStr">
-        <is>
-          <t>University Campus Study Lounge</t>
+          <t>No</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Moderate Student &amp; Academic</t>
+          <t>High</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Economical / Low Overhead ($)</t>
+          <t>Affordable</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Extended Study &amp; Work (&gt; 60 mins)</t>
+          <t>Low</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>Transit Hub / Walk-Up Only (Zero Parking)</t>
+          <t>Poor</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>Standard Lounge (80 - 150 sqm)</t>
-        </is>
-      </c>
-      <c r="F8" t="inlineStr">
-        <is>
-          <t>University Campus Study Lounge</t>
+          <t>No</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Moderate Student &amp; Academic</t>
+          <t>Moderate</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Moderate / Urban Commercial ($$)</t>
+          <t>Affordable</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Extended Study &amp; Work (&gt; 60 mins)</t>
+          <t>Low</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>Street Parking &amp; Shared Lot</t>
+          <t>Good</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>Spacious Destination (&gt; 200 sqm)</t>
-        </is>
-      </c>
-      <c r="F9" t="inlineStr">
-        <is>
-          <t>University Campus Study Lounge</t>
+          <t>Yes</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Moderate Student &amp; Academic</t>
+          <t>Moderate</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Economical / Low Overhead ($)</t>
+          <t>Affordable</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Extended Study &amp; Work (&gt; 60 mins)</t>
+          <t>High</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>Street Parking &amp; Shared Lot</t>
+          <t>Good</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>Standard Lounge (80 - 150 sqm)</t>
-        </is>
-      </c>
-      <c r="F10" t="inlineStr">
-        <is>
-          <t>University Campus Study Lounge</t>
+          <t>No</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Neighborhood Residents &amp; Families</t>
+          <t>Moderate</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Moderate / Urban Commercial ($$)</t>
+          <t>Moderate</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Social Dine-In &amp; Brunch (30 - 60 mins)</t>
+          <t>Low</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>Street Parking &amp; Shared Lot</t>
+          <t>Good</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>Spacious Destination (&gt; 200 sqm)</t>
-        </is>
-      </c>
-      <c r="F11" t="inlineStr">
-        <is>
-          <t>Suburban Community Roastery &amp; Patio</t>
+          <t>Yes</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Neighborhood Residents &amp; Families</t>
+          <t>Moderate</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Economical / Low Overhead ($)</t>
+          <t>Moderate</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Social Dine-In &amp; Brunch (30 - 60 mins)</t>
+          <t>High</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>Street Parking &amp; Shared Lot</t>
+          <t>Good</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>Spacious Destination (&gt; 200 sqm)</t>
-        </is>
-      </c>
-      <c r="F12" t="inlineStr">
-        <is>
-          <t>Suburban Community Roastery &amp; Patio</t>
+          <t>No</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Neighborhood Residents &amp; Families</t>
+          <t>Moderate</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Moderate / Urban Commercial ($$)</t>
+          <t>Expensive</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Social Dine-In &amp; Brunch (30 - 60 mins)</t>
+          <t>Low</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>Street Parking &amp; Shared Lot</t>
+          <t>Good</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>Standard Lounge (80 - 150 sqm)</t>
-        </is>
-      </c>
-      <c r="F13" t="inlineStr">
-        <is>
-          <t>Suburban Community Roastery &amp; Patio</t>
+          <t>No</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Neighborhood Residents &amp; Families</t>
+          <t>Moderate</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Moderate / Urban Commercial ($$)</t>
+          <t>Affordable</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Extended Study &amp; Work (&gt; 60 mins)</t>
+          <t>Low</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>Street Parking &amp; Shared Lot</t>
+          <t>Poor</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>Spacious Destination (&gt; 200 sqm)</t>
-        </is>
-      </c>
-      <c r="F14" t="inlineStr">
-        <is>
-          <t>Suburban Community Roastery &amp; Patio</t>
+          <t>No</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Neighborhood Residents &amp; Families</t>
+          <t>Low</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Economical / Low Overhead ($)</t>
+          <t>Affordable</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Social Dine-In &amp; Brunch (30 - 60 mins)</t>
+          <t>Low</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>Dedicated Drive-Thru &amp; Ample Parking</t>
+          <t>Good</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>Spacious Destination (&gt; 200 sqm)</t>
-        </is>
-      </c>
-      <c r="F15" t="inlineStr">
-        <is>
-          <t>Suburban Community Roastery &amp; Patio</t>
+          <t>No</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Low Pedestrian / High Vehicular Flow</t>
+          <t>Low</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Economical / Low Overhead ($)</t>
+          <t>Affordable</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Grab-&amp;-Go (&lt; 10 mins)</t>
+          <t>High</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>Dedicated Drive-Thru &amp; Ample Parking</t>
+          <t>Poor</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>Standard Lounge (80 - 150 sqm)</t>
-        </is>
-      </c>
-      <c r="F16" t="inlineStr">
-        <is>
-          <t>Highway Commuter Drive-Thru Express</t>
+          <t>No</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Low Pedestrian / High Vehicular Flow</t>
+          <t>Low</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Moderate / Urban Commercial ($$)</t>
+          <t>Moderate</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>Grab-&amp;-Go (&lt; 10 mins)</t>
+          <t>Low</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>Dedicated Drive-Thru &amp; Ample Parking</t>
+          <t>Good</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>Standard Lounge (80 - 150 sqm)</t>
-        </is>
-      </c>
-      <c r="F17" t="inlineStr">
-        <is>
-          <t>Highway Commuter Drive-Thru Express</t>
+          <t>No</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Low Pedestrian / High Vehicular Flow</t>
+          <t>Low</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Economical / Low Overhead ($)</t>
+          <t>Expensive</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>Grab-&amp;-Go (&lt; 10 mins)</t>
+          <t>Low</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>Dedicated Drive-Thru &amp; Ample Parking</t>
+          <t>Poor</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>Micro Space (&lt; 40 sqm)</t>
-        </is>
-      </c>
-      <c r="F18" t="inlineStr">
-        <is>
-          <t>Highway Commuter Drive-Thru Express</t>
-        </is>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" t="inlineStr">
-        <is>
-          <t>Low Pedestrian / High Vehicular Flow</t>
-        </is>
-      </c>
-      <c r="B19" t="inlineStr">
-        <is>
-          <t>Economical / Low Overhead ($)</t>
-        </is>
-      </c>
-      <c r="C19" t="inlineStr">
-        <is>
-          <t>Social Dine-In &amp; Brunch (30 - 60 mins)</t>
-        </is>
-      </c>
-      <c r="D19" t="inlineStr">
-        <is>
-          <t>Dedicated Drive-Thru &amp; Ample Parking</t>
-        </is>
-      </c>
-      <c r="E19" t="inlineStr">
-        <is>
-          <t>Standard Lounge (80 - 150 sqm)</t>
-        </is>
-      </c>
-      <c r="F19" t="inlineStr">
-        <is>
-          <t>Highway Commuter Drive-Thru Express</t>
-        </is>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" t="inlineStr">
-        <is>
-          <t>Weekend Leisure &amp; Tourists</t>
-        </is>
-      </c>
-      <c r="B20" t="inlineStr">
-        <is>
-          <t>High / Prime Downtown ($$$$)</t>
-        </is>
-      </c>
-      <c r="C20" t="inlineStr">
-        <is>
-          <t>Social Dine-In &amp; Brunch (30 - 60 mins)</t>
-        </is>
-      </c>
-      <c r="D20" t="inlineStr">
-        <is>
-          <t>Transit Hub / Walk-Up Only (Zero Parking)</t>
-        </is>
-      </c>
-      <c r="E20" t="inlineStr">
-        <is>
-          <t>Spacious Destination (&gt; 200 sqm)</t>
-        </is>
-      </c>
-      <c r="F20" t="inlineStr">
-        <is>
-          <t>Arts &amp; Heritage Flagship Tasting Room</t>
-        </is>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" t="inlineStr">
-        <is>
-          <t>Weekend Leisure &amp; Tourists</t>
-        </is>
-      </c>
-      <c r="B21" t="inlineStr">
-        <is>
-          <t>Moderate / Urban Commercial ($$)</t>
-        </is>
-      </c>
-      <c r="C21" t="inlineStr">
-        <is>
-          <t>Social Dine-In &amp; Brunch (30 - 60 mins)</t>
-        </is>
-      </c>
-      <c r="D21" t="inlineStr">
-        <is>
-          <t>Street Parking &amp; Shared Lot</t>
-        </is>
-      </c>
-      <c r="E21" t="inlineStr">
-        <is>
-          <t>Spacious Destination (&gt; 200 sqm)</t>
-        </is>
-      </c>
-      <c r="F21" t="inlineStr">
-        <is>
-          <t>Arts &amp; Heritage Flagship Tasting Room</t>
-        </is>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" t="inlineStr">
-        <is>
-          <t>Weekend Leisure &amp; Tourists</t>
-        </is>
-      </c>
-      <c r="B22" t="inlineStr">
-        <is>
-          <t>High / Prime Downtown ($$$$)</t>
-        </is>
-      </c>
-      <c r="C22" t="inlineStr">
-        <is>
-          <t>Extended Study &amp; Work (&gt; 60 mins)</t>
-        </is>
-      </c>
-      <c r="D22" t="inlineStr">
-        <is>
-          <t>Street Parking &amp; Shared Lot</t>
-        </is>
-      </c>
-      <c r="E22" t="inlineStr">
-        <is>
-          <t>Spacious Destination (&gt; 200 sqm)</t>
-        </is>
-      </c>
-      <c r="F22" t="inlineStr">
-        <is>
-          <t>Arts &amp; Heritage Flagship Tasting Room</t>
-        </is>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" t="inlineStr">
-        <is>
-          <t>Weekend Leisure &amp; Tourists</t>
-        </is>
-      </c>
-      <c r="B23" t="inlineStr">
-        <is>
-          <t>Moderate / Urban Commercial ($$)</t>
-        </is>
-      </c>
-      <c r="C23" t="inlineStr">
-        <is>
-          <t>Extended Study &amp; Work (&gt; 60 mins)</t>
-        </is>
-      </c>
-      <c r="D23" t="inlineStr">
-        <is>
-          <t>Transit Hub / Walk-Up Only (Zero Parking)</t>
-        </is>
-      </c>
-      <c r="E23" t="inlineStr">
-        <is>
-          <t>Spacious Destination (&gt; 200 sqm)</t>
-        </is>
-      </c>
-      <c r="F23" t="inlineStr">
-        <is>
-          <t>Arts &amp; Heritage Flagship Tasting Room</t>
-        </is>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" t="inlineStr">
-        <is>
-          <t>Heavy Transit &amp; Office Commuters</t>
-        </is>
-      </c>
-      <c r="B24" t="inlineStr">
-        <is>
-          <t>Economical / Low Overhead ($)</t>
-        </is>
-      </c>
-      <c r="C24" t="inlineStr">
-        <is>
-          <t>Grab-&amp;-Go (&lt; 10 mins)</t>
-        </is>
-      </c>
-      <c r="D24" t="inlineStr">
-        <is>
-          <t>Street Parking &amp; Shared Lot</t>
-        </is>
-      </c>
-      <c r="E24" t="inlineStr">
-        <is>
-          <t>Micro Space (&lt; 40 sqm)</t>
-        </is>
-      </c>
-      <c r="F24" t="inlineStr">
-        <is>
-          <t>Corporate Business Park Micro-Lobby</t>
-        </is>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" t="inlineStr">
-        <is>
-          <t>Heavy Transit &amp; Office Commuters</t>
-        </is>
-      </c>
-      <c r="B25" t="inlineStr">
-        <is>
-          <t>Economical / Low Overhead ($)</t>
-        </is>
-      </c>
-      <c r="C25" t="inlineStr">
-        <is>
-          <t>Grab-&amp;-Go (&lt; 10 mins)</t>
-        </is>
-      </c>
-      <c r="D25" t="inlineStr">
-        <is>
-          <t>Transit Hub / Walk-Up Only (Zero Parking)</t>
-        </is>
-      </c>
-      <c r="E25" t="inlineStr">
-        <is>
-          <t>Micro Space (&lt; 40 sqm)</t>
-        </is>
-      </c>
-      <c r="F25" t="inlineStr">
-        <is>
-          <t>Corporate Business Park Micro-Lobby</t>
-        </is>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" t="inlineStr">
-        <is>
-          <t>Moderate Student &amp; Academic</t>
-        </is>
-      </c>
-      <c r="B26" t="inlineStr">
-        <is>
-          <t>Economical / Low Overhead ($)</t>
-        </is>
-      </c>
-      <c r="C26" t="inlineStr">
-        <is>
-          <t>Grab-&amp;-Go (&lt; 10 mins)</t>
-        </is>
-      </c>
-      <c r="D26" t="inlineStr">
-        <is>
-          <t>Transit Hub / Walk-Up Only (Zero Parking)</t>
-        </is>
-      </c>
-      <c r="E26" t="inlineStr">
-        <is>
-          <t>Micro Space (&lt; 40 sqm)</t>
-        </is>
-      </c>
-      <c r="F26" t="inlineStr">
-        <is>
-          <t>Corporate Business Park Micro-Lobby</t>
-        </is>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27" t="inlineStr">
-        <is>
-          <t>Heavy Transit &amp; Office Commuters</t>
-        </is>
-      </c>
-      <c r="B27" t="inlineStr">
-        <is>
-          <t>Economical / Low Overhead ($)</t>
-        </is>
-      </c>
-      <c r="C27" t="inlineStr">
-        <is>
-          <t>Moderate Stay (15 - 45 mins)</t>
-        </is>
-      </c>
-      <c r="D27" t="inlineStr">
-        <is>
-          <t>Street Parking &amp; Shared Lot</t>
-        </is>
-      </c>
-      <c r="E27" t="inlineStr">
-        <is>
-          <t>Micro Space (&lt; 40 sqm)</t>
-        </is>
-      </c>
-      <c r="F27" t="inlineStr">
-        <is>
-          <t>Corporate Business Park Micro-Lobby</t>
+          <t>No</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat: upgrade Decision Tree to professional retail acquisition feasibility engine (YES/NO)
</commit_message>
<xml_diff>
--- a/data/RoastLab_All_Datasets.xlsx
+++ b/data/RoastLab_All_Datasets.xlsx
@@ -25605,7 +25605,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E18"/>
+  <dimension ref="A1:E22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -25616,481 +25616,589 @@
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>rent_cost</t>
+          <t>lease_overhead</t>
         </is>
       </c>
       <c r="C1" t="inlineStr">
         <is>
-          <t>competition</t>
+          <t>competition_density</t>
         </is>
       </c>
       <c r="D1" t="inlineStr">
         <is>
-          <t>accessibility</t>
+          <t>transit_access</t>
         </is>
       </c>
       <c r="E1" t="inlineStr">
         <is>
-          <t>open_coffee_shop</t>
+          <t>expansion_verdict</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>High Volume (&gt; 15k pedestrians/day)</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Affordable</t>
+          <t>Favorable (&lt; 10% revenue)</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Low</t>
+          <t>Low Saturation (0-2 cafes)</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Good</t>
+          <t>Prime Accessibility (Transit Hub)</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>YES</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>High Volume (&gt; 15k pedestrians/day)</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Affordable</t>
+          <t>Favorable (&lt; 10% revenue)</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Moderate Saturation (3-5 cafes)</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Good</t>
+          <t>Prime Accessibility (Transit Hub)</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>YES</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>High Volume (&gt; 15k pedestrians/day)</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Moderate</t>
+          <t>Favorable (&lt; 10% revenue)</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Low</t>
+          <t>Heavy Saturation (&gt; 5 cafes)</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Good</t>
+          <t>Prime Accessibility (Transit Hub)</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>YES</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>High Volume (&gt; 15k pedestrians/day)</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Moderate</t>
+          <t>Moderate Market Rate (10-18%)</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Low Saturation (0-2 cafes)</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Good</t>
+          <t>Prime Accessibility (Transit Hub)</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>YES</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>High Volume (&gt; 15k pedestrians/day)</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Expensive</t>
+          <t>Moderate Market Rate (10-18%)</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Low</t>
+          <t>Moderate Saturation (3-5 cafes)</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>Good</t>
+          <t>Prime Accessibility (Transit Hub)</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>YES</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>High Volume (&gt; 15k pedestrians/day)</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Expensive</t>
+          <t>Moderate Market Rate (10-18%)</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Heavy Saturation (&gt; 5 cafes)</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>Good</t>
+          <t>Prime Accessibility (Transit Hub)</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>YES</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>High Volume (&gt; 15k pedestrians/day)</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Affordable</t>
+          <t>Prime / Premium Overhead (&gt; 18%)</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Low</t>
+          <t>Low Saturation (0-2 cafes)</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>Poor</t>
+          <t>Prime Accessibility (Transit Hub)</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>YES</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Moderate</t>
+          <t>High Volume (&gt; 15k pedestrians/day)</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Affordable</t>
+          <t>Prime / Premium Overhead (&gt; 18%)</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Low</t>
+          <t>Heavy Saturation (&gt; 5 cafes)</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>Good</t>
+          <t>Prime Accessibility (Transit Hub)</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>NO</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Moderate</t>
+          <t>High Volume (&gt; 15k pedestrians/day)</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Affordable</t>
+          <t>Favorable (&lt; 10% revenue)</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Low Saturation (0-2 cafes)</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>Good</t>
+          <t>Restricted (Poor Walkability)</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>NO</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Moderate</t>
+          <t>Moderate Volume (5k-15k pedestrians/day)</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Moderate</t>
+          <t>Favorable (&lt; 10% revenue)</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Low</t>
+          <t>Low Saturation (0-2 cafes)</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>Good</t>
+          <t>Prime Accessibility (Transit Hub)</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>YES</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Moderate</t>
+          <t>Moderate Volume (5k-15k pedestrians/day)</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Moderate</t>
+          <t>Favorable (&lt; 10% revenue)</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Moderate Saturation (3-5 cafes)</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>Good</t>
+          <t>Standard Accessibility (Streetflow)</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>YES</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Moderate</t>
+          <t>Moderate Volume (5k-15k pedestrians/day)</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Expensive</t>
+          <t>Favorable (&lt; 10% revenue)</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Low</t>
+          <t>Heavy Saturation (&gt; 5 cafes)</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>Good</t>
+          <t>Standard Accessibility (Streetflow)</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>NO</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Moderate</t>
+          <t>Moderate Volume (5k-15k pedestrians/day)</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Affordable</t>
+          <t>Moderate Market Rate (10-18%)</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Low</t>
+          <t>Low Saturation (0-2 cafes)</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>Poor</t>
+          <t>Standard Accessibility (Streetflow)</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>YES</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Low</t>
+          <t>Moderate Volume (5k-15k pedestrians/day)</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Affordable</t>
+          <t>Moderate Market Rate (10-18%)</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Low</t>
+          <t>Moderate Saturation (3-5 cafes)</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>Good</t>
+          <t>Standard Accessibility (Streetflow)</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>YES</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Low</t>
+          <t>Moderate Volume (5k-15k pedestrians/day)</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Affordable</t>
+          <t>Moderate Market Rate (10-18%)</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Heavy Saturation (&gt; 5 cafes)</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>Poor</t>
+          <t>Standard Accessibility (Streetflow)</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>NO</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Low</t>
+          <t>Moderate Volume (5k-15k pedestrians/day)</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Moderate</t>
+          <t>Prime / Premium Overhead (&gt; 18%)</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>Low</t>
+          <t>Low Saturation (0-2 cafes)</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>Good</t>
+          <t>Standard Accessibility (Streetflow)</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>NO</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Low</t>
+          <t>Moderate Volume (5k-15k pedestrians/day)</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Expensive</t>
+          <t>Moderate Market Rate (10-18%)</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>Low</t>
+          <t>Low Saturation (0-2 cafes)</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>Poor</t>
+          <t>Restricted (Poor Walkability)</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>NO</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>Low Volume (&lt; 5k pedestrians/day)</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>Favorable (&lt; 10% revenue)</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>Low Saturation (0-2 cafes)</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>Standard Accessibility (Streetflow)</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>Low Volume (&lt; 5k pedestrians/day)</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>Favorable (&lt; 10% revenue)</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>Heavy Saturation (&gt; 5 cafes)</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>Restricted (Poor Walkability)</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>Low Volume (&lt; 5k pedestrians/day)</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>Moderate Market Rate (10-18%)</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>Low Saturation (0-2 cafes)</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>Standard Accessibility (Streetflow)</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>Low Volume (&lt; 5k pedestrians/day)</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>Prime / Premium Overhead (&gt; 18%)</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>Low Saturation (0-2 cafes)</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>Restricted (Poor Walkability)</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>NO</t>
         </is>
       </c>
     </row>

</xml_diff>